<commit_message>
Deploying to gh-pages from @ tarun2184/DEVLINK@993a56d2694ef1c3d21bd28676e87984e7a094ce 🚀
</commit_message>
<xml_diff>
--- a/reports/Performance_Load_Test_Report.xlsx
+++ b/reports/Performance_Load_Test_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="163">
   <si>
     <t>Test ID</t>
   </si>
@@ -43,7 +43,7 @@
     <t>Baseline 100 VUs</t>
   </si>
   <si>
-    <t>Load Test Request Execution #1 (Target: /DEVLINK/)</t>
+    <t>k6 Performance Request Execution #1 (Target: /DEVLINK/)</t>
   </si>
   <si>
     <t>k6 Load Tester</t>
@@ -52,364 +52,454 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-08-07T03:44:46.925Z</t>
-  </si>
-  <si>
-    <t>Response latency 221.41ms (Threshold: &lt; 1500ms)</t>
+    <t>2026-08-07T03:50:25.848Z</t>
+  </si>
+  <si>
+    <t>Response latency 177.85ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-002</t>
   </si>
   <si>
-    <t>Load Test Request Execution #2 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 206.12ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #2 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 141.24ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-003</t>
   </si>
   <si>
-    <t>Load Test Request Execution #3 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 161.90ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #3 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 89.31ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-004</t>
   </si>
   <si>
-    <t>Load Test Request Execution #4 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 150.67ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #4 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 119.03ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-005</t>
   </si>
   <si>
-    <t>Load Test Request Execution #5 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 167.86ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #5 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 205.90ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-006</t>
   </si>
   <si>
-    <t>Load Test Request Execution #6 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 192.69ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #6 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 80.71ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-007</t>
   </si>
   <si>
-    <t>Load Test Request Execution #7 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 219.75ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #7 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 188.73ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-008</t>
   </si>
   <si>
-    <t>Load Test Request Execution #8 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 248.14ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #8 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 91.11ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-009</t>
   </si>
   <si>
-    <t>Load Test Request Execution #9 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 96.12ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #9 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 163.00ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-010</t>
   </si>
   <si>
-    <t>Load Test Request Execution #10 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 75.29ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #10 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 193.04ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-011</t>
   </si>
   <si>
-    <t>Load Test Request Execution #11 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 121.21ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #11 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 133.42ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-012</t>
   </si>
   <si>
-    <t>Load Test Request Execution #12 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 121.84ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #12 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 132.60ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-013</t>
   </si>
   <si>
-    <t>Load Test Request Execution #13 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 243.44ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #13 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 177.50ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-014</t>
   </si>
   <si>
-    <t>Load Test Request Execution #14 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 139.53ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #14 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 180.43ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-015</t>
   </si>
   <si>
-    <t>Load Test Request Execution #15 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 97.43ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #15 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 102.01ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-016</t>
   </si>
   <si>
-    <t>Load Test Request Execution #16 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 145.14ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #16 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 216.37ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-017</t>
   </si>
   <si>
-    <t>Load Test Request Execution #17 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 173.03ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #17 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 78.36ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-018</t>
   </si>
   <si>
-    <t>Load Test Request Execution #18 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 165.37ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #18 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 72.34ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-019</t>
   </si>
   <si>
-    <t>Load Test Request Execution #19 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 68.71ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #19 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 166.36ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-020</t>
   </si>
   <si>
-    <t>Load Test Request Execution #20 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 240.47ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #20 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 224.13ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-021</t>
   </si>
   <si>
-    <t>Spike &amp; Stress 200 VUs</t>
-  </si>
-  <si>
-    <t>Load Test Request Execution #21 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 127.68ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #21 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 72.49ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-022</t>
   </si>
   <si>
-    <t>Load Test Request Execution #22 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 117.33ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #22 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 73.94ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-023</t>
   </si>
   <si>
-    <t>Load Test Request Execution #23 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 243.69ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #23 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 202.48ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-024</t>
   </si>
   <si>
-    <t>Load Test Request Execution #24 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 145.17ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #24 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 76.22ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-025</t>
   </si>
   <si>
-    <t>Load Test Request Execution #25 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 213.91ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #25 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 190.97ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-026</t>
   </si>
   <si>
-    <t>Load Test Request Execution #26 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 111.25ms (Threshold: &lt; 1500ms)</t>
+    <t>Spike &amp; Load 150 VUs</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #26 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 158.51ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-027</t>
   </si>
   <si>
-    <t>Load Test Request Execution #27 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 55.72ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #27 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 108.01ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-028</t>
   </si>
   <si>
-    <t>Load Test Request Execution #28 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 227.09ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #28 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 187.21ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-029</t>
   </si>
   <si>
-    <t>Load Test Request Execution #29 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 130.39ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #29 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 154.40ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-030</t>
   </si>
   <si>
-    <t>Load Test Request Execution #30 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 168.73ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #30 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 212.05ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-031</t>
   </si>
   <si>
-    <t>Load Test Request Execution #31 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 63.17ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #31 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 70.86ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-032</t>
   </si>
   <si>
-    <t>Load Test Request Execution #32 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 65.41ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #32 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 64.24ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-033</t>
   </si>
   <si>
-    <t>Load Test Request Execution #33 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 101.10ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #33 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 83.79ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-034</t>
   </si>
   <si>
-    <t>Load Test Request Execution #34 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 215.86ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #34 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 169.00ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-035</t>
   </si>
   <si>
-    <t>Load Test Request Execution #35 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 151.10ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #35 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 198.90ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-036</t>
   </si>
   <si>
-    <t>Load Test Request Execution #36 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 164.03ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #36 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 55.77ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-037</t>
   </si>
   <si>
-    <t>Load Test Request Execution #37 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 114.12ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #37 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 92.51ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-038</t>
   </si>
   <si>
-    <t>Load Test Request Execution #38 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 53.15ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #38 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 74.50ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-039</t>
   </si>
   <si>
-    <t>Load Test Request Execution #39 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 78.78ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #39 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 115.28ms (Threshold: &lt; 1500ms)</t>
   </si>
   <si>
     <t>PERF-TC-040</t>
   </si>
   <si>
-    <t>Load Test Request Execution #40 (Target: /DEVLINK/)</t>
-  </si>
-  <si>
-    <t>Response latency 89.96ms (Threshold: &lt; 1500ms)</t>
+    <t>k6 Performance Request Execution #40 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 176.57ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-041</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #41 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 132.74ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-042</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #42 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 211.99ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-043</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #43 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 114.58ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-044</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #44 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 150.31ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-045</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #45 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 70.75ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-046</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #46 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 180.81ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-047</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #47 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 219.98ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-048</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #48 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 121.41ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-049</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #49 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 54.85ms (Threshold: &lt; 1500ms)</t>
+  </si>
+  <si>
+    <t>PERF-TC-050</t>
+  </si>
+  <si>
+    <t>k6 Performance Request Execution #50 (Target: /DEVLINK/)</t>
+  </si>
+  <si>
+    <t>Response latency 191.82ms (Threshold: &lt; 1500ms)</t>
   </si>
 </sst>
 </file>
@@ -851,12 +941,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
@@ -904,7 +994,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2">
-        <v>221.41</v>
+        <v>177.85</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>12</v>
@@ -930,7 +1020,7 @@
         <v>11</v>
       </c>
       <c r="E3" s="4">
-        <v>206.12</v>
+        <v>141.24</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>12</v>
@@ -956,7 +1046,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="2">
-        <v>161.9</v>
+        <v>89.31</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>12</v>
@@ -982,7 +1072,7 @@
         <v>11</v>
       </c>
       <c r="E5" s="4">
-        <v>150.67</v>
+        <v>119.03</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>12</v>
@@ -1008,7 +1098,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="2">
-        <v>167.86</v>
+        <v>205.9</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>12</v>
@@ -1034,7 +1124,7 @@
         <v>11</v>
       </c>
       <c r="E7" s="4">
-        <v>192.69</v>
+        <v>80.71</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>12</v>
@@ -1060,7 +1150,7 @@
         <v>11</v>
       </c>
       <c r="E8" s="2">
-        <v>219.75</v>
+        <v>188.73</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>12</v>
@@ -1086,7 +1176,7 @@
         <v>11</v>
       </c>
       <c r="E9" s="4">
-        <v>248.14</v>
+        <v>91.11</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>12</v>
@@ -1112,7 +1202,7 @@
         <v>11</v>
       </c>
       <c r="E10" s="2">
-        <v>96.12</v>
+        <v>163</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>12</v>
@@ -1138,7 +1228,7 @@
         <v>11</v>
       </c>
       <c r="E11" s="4">
-        <v>75.29</v>
+        <v>193.04</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>12</v>
@@ -1164,7 +1254,7 @@
         <v>11</v>
       </c>
       <c r="E12" s="2">
-        <v>121.21</v>
+        <v>133.42</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>12</v>
@@ -1190,7 +1280,7 @@
         <v>11</v>
       </c>
       <c r="E13" s="4">
-        <v>121.84</v>
+        <v>132.6</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>12</v>
@@ -1216,7 +1306,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="2">
-        <v>243.44</v>
+        <v>177.5</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>12</v>
@@ -1242,7 +1332,7 @@
         <v>11</v>
       </c>
       <c r="E15" s="4">
-        <v>139.53</v>
+        <v>180.43</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>12</v>
@@ -1268,7 +1358,7 @@
         <v>11</v>
       </c>
       <c r="E16" s="2">
-        <v>97.43</v>
+        <v>102.01</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>12</v>
@@ -1294,7 +1384,7 @@
         <v>11</v>
       </c>
       <c r="E17" s="4">
-        <v>145.14</v>
+        <v>216.37</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>12</v>
@@ -1320,7 +1410,7 @@
         <v>11</v>
       </c>
       <c r="E18" s="2">
-        <v>173.03</v>
+        <v>78.36</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>12</v>
@@ -1346,7 +1436,7 @@
         <v>11</v>
       </c>
       <c r="E19" s="4">
-        <v>165.37</v>
+        <v>72.34</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>12</v>
@@ -1372,7 +1462,7 @@
         <v>11</v>
       </c>
       <c r="E20" s="2">
-        <v>68.71</v>
+        <v>166.36</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>12</v>
@@ -1398,7 +1488,7 @@
         <v>11</v>
       </c>
       <c r="E21" s="4">
-        <v>240.47</v>
+        <v>224.13</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>12</v>
@@ -1415,137 +1505,137 @@
         <v>72</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="2">
+        <v>72.49</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" s="2">
-        <v>127.68</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" s="4">
+        <v>73.94</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" s="4">
-        <v>117.33</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="2">
+        <v>202.48</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" s="2">
-        <v>243.69</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="4" t="s">
+      <c r="D25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" s="4">
+        <v>76.22</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" s="4">
-        <v>145.17</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="2">
+        <v>190.97</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" s="2">
-        <v>213.91</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>89</v>
@@ -1554,7 +1644,7 @@
         <v>11</v>
       </c>
       <c r="E27" s="4">
-        <v>111.25</v>
+        <v>158.51</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>12</v>
@@ -1571,7 +1661,7 @@
         <v>91</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>92</v>
@@ -1580,7 +1670,7 @@
         <v>11</v>
       </c>
       <c r="E28" s="2">
-        <v>55.72</v>
+        <v>108.01</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>12</v>
@@ -1597,7 +1687,7 @@
         <v>94</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>95</v>
@@ -1606,7 +1696,7 @@
         <v>11</v>
       </c>
       <c r="E29" s="4">
-        <v>227.09</v>
+        <v>187.21</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>12</v>
@@ -1623,7 +1713,7 @@
         <v>97</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>98</v>
@@ -1632,7 +1722,7 @@
         <v>11</v>
       </c>
       <c r="E30" s="2">
-        <v>130.39</v>
+        <v>154.4</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>12</v>
@@ -1649,7 +1739,7 @@
         <v>100</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>101</v>
@@ -1658,7 +1748,7 @@
         <v>11</v>
       </c>
       <c r="E31" s="4">
-        <v>168.73</v>
+        <v>212.05</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>12</v>
@@ -1675,7 +1765,7 @@
         <v>103</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>104</v>
@@ -1684,7 +1774,7 @@
         <v>11</v>
       </c>
       <c r="E32" s="2">
-        <v>63.17</v>
+        <v>70.86</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>12</v>
@@ -1701,7 +1791,7 @@
         <v>106</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>107</v>
@@ -1710,7 +1800,7 @@
         <v>11</v>
       </c>
       <c r="E33" s="4">
-        <v>65.41</v>
+        <v>64.24</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>12</v>
@@ -1727,7 +1817,7 @@
         <v>109</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>110</v>
@@ -1736,7 +1826,7 @@
         <v>11</v>
       </c>
       <c r="E34" s="2">
-        <v>101.1</v>
+        <v>83.79</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>12</v>
@@ -1753,7 +1843,7 @@
         <v>112</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>113</v>
@@ -1762,7 +1852,7 @@
         <v>11</v>
       </c>
       <c r="E35" s="4">
-        <v>215.86</v>
+        <v>169</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>12</v>
@@ -1779,7 +1869,7 @@
         <v>115</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>116</v>
@@ -1788,7 +1878,7 @@
         <v>11</v>
       </c>
       <c r="E36" s="2">
-        <v>151.1</v>
+        <v>198.9</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>12</v>
@@ -1805,7 +1895,7 @@
         <v>118</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>119</v>
@@ -1814,7 +1904,7 @@
         <v>11</v>
       </c>
       <c r="E37" s="4">
-        <v>164.03</v>
+        <v>55.77</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>12</v>
@@ -1831,7 +1921,7 @@
         <v>121</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>122</v>
@@ -1840,7 +1930,7 @@
         <v>11</v>
       </c>
       <c r="E38" s="2">
-        <v>114.12</v>
+        <v>92.51</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>12</v>
@@ -1857,7 +1947,7 @@
         <v>124</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>125</v>
@@ -1866,7 +1956,7 @@
         <v>11</v>
       </c>
       <c r="E39" s="4">
-        <v>53.15</v>
+        <v>74.5</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>12</v>
@@ -1883,7 +1973,7 @@
         <v>127</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>128</v>
@@ -1892,7 +1982,7 @@
         <v>11</v>
       </c>
       <c r="E40" s="2">
-        <v>78.78</v>
+        <v>115.28</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>12</v>
@@ -1909,7 +1999,7 @@
         <v>130</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>131</v>
@@ -1918,7 +2008,7 @@
         <v>11</v>
       </c>
       <c r="E41" s="4">
-        <v>89.96</v>
+        <v>176.57</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>12</v>
@@ -1928,6 +2018,266 @@
       </c>
       <c r="H41" s="4" t="s">
         <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" s="2">
+        <v>132.74</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" s="4">
+        <v>211.99</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" s="2">
+        <v>114.58</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" s="4">
+        <v>150.31</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" s="2">
+        <v>70.75</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="4">
+        <v>180.81</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="2">
+        <v>219.98</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="4">
+        <v>121.41</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="2">
+        <v>54.85</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" s="4">
+        <v>191.82</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>